<commit_message>
Add private three-quiz assessment and teacher-approved class grouping
</commit_message>
<xml_diff>
--- a/public/student-template.xlsx
+++ b/public/student-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\我的文档\作业+论文+文件\2026-09-15陈辉毕业设计平台\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC526AB-4EB4-460A-91C7-1274788FCF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04AEF31C-A63E-4F4D-A96F-C8B45296D580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>姓名</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -36,6 +36,26 @@
   </si>
   <si>
     <t>性别</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>班级</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>张三</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>男</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>八年级1班</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>（例子填写时需删除）</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -43,7 +63,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -53,6 +73,21 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -79,8 +114,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -361,10 +402,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -373,6 +417,26 @@
       </c>
       <c r="C1" t="s">
         <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polish refresh icon and update student template
</commit_message>
<xml_diff>
--- a/public/student-template.xlsx
+++ b/public/student-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\我的文档\作业+论文+文件\2026-09-15陈辉毕业设计平台\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04AEF31C-A63E-4F4D-A96F-C8B45296D580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64AD647D-589D-4AA3-B6C9-885149250312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>（例子填写时需删除）</t>
+    <t>（请严格按照例子格式填写，否则会报错！！！！实际填写时请删除这一行）</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -405,7 +405,7 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="67.4140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Refine class-scoped assessment records
</commit_message>
<xml_diff>
--- a/public/student-template.xlsx
+++ b/public/student-template.xlsx
@@ -1,97 +1,68 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\我的文档\作业+论文+文件\2026-09-15陈辉毕业设计平台\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64AD647D-589D-4AA3-B6C9-885149250312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>姓名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>年龄</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>性别</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>班级</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>张三</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>男</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>八年级1班</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>（请严格按照例子格式填写，否则会报错！！！！实际填写时请删除这一行）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
       <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
+      <charset val="134"/>
+      <color rgb="FFFF0000"/>
+      <family val="3"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="等线"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -116,15 +87,15 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -401,47 +372,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
-    <col min="5" max="5" width="67.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="2">
-        <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>7</v>
-      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>